<commit_message>
Usa la fuente definitiva de El sin por qué del destino
</commit_message>
<xml_diff>
--- a/outputs/fechas/fechas.xlsx
+++ b/outputs/fechas/fechas.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fechas" sheetId="1" r:id="R762c6bee52144deb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fechas" sheetId="1" r:id="R852e2a158b9d441d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1437,14 +1437,14 @@
       <x:c r="D50" s="11"/>
       <x:c r="E50" s="12" t="str"/>
       <x:c r="F50" s="12" t="str">
-        <x:v>fecha_modificacion</x:v>
+        <x:v>fecha_de_los_fragmentos_originales</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str"/>
       <x:c r="H50" s="15" t="n">
         <x:v>38646.708333333336</x:v>
       </x:c>
       <x:c r="I50" s="13" t="str">
-        <x:v>poesias/imagenes/el sin por que del destino 1-4.txt</x:v>
+        <x:v>poesias/imagenes/el sin por que del destino definitivo.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
@@ -2198,7 +2198,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9794c73b49c94b59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2715403a439d4ea0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>